<commit_message>
nmv 29 04 2026
</commit_message>
<xml_diff>
--- a/TS Jatai Working/Padam Input Templates/TS 1.3 Padam Input Template.xlsx
+++ b/TS Jatai Working/Padam Input Templates/TS 1.3 Padam Input Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ALL IMP DATA\GitHub\texts\TS Jatai Working\Padam Input Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ECA6263-0480-43DE-B601-3AC64BAAEC03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F70885C-30C2-44C6-B071-D41F752ADFDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3757,9 +3757,6 @@
   </si>
   <si>
     <t xml:space="preserve">puqruqspRuhaqmiti# puru - spRuha$m </t>
-  </si>
-  <si>
-    <t xml:space="preserve">raqyimiti# rayim </t>
   </si>
   <si>
     <t xml:space="preserve">roqcaqnaqsthA iti# rocana - sthAH </t>
@@ -4078,6 +4075,9 @@
   </si>
   <si>
     <t xml:space="preserve">aqreqpasAqvitya#reqpasau$ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">raqyimiti# raqyim </t>
   </si>
 </sst>
 </file>
@@ -5219,7 +5219,7 @@
   <sheetData>
     <row r="1" spans="1:22" ht="72" x14ac:dyDescent="0.25">
       <c r="A1" s="50" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15" t="s">
@@ -5271,10 +5271,10 @@
         <v>10</v>
       </c>
       <c r="S1" s="39" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
       <c r="T1" s="39" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
       <c r="U1" s="38" t="s">
         <v>17</v>
@@ -5425,7 +5425,7 @@
         <v>4</v>
       </c>
       <c r="N5" s="8" t="s">
-        <v>1303</v>
+        <v>1302</v>
       </c>
       <c r="O5" s="2" t="s">
         <v>0</v>
@@ -13105,7 +13105,7 @@
     </row>
     <row r="264" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A264" s="51" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
       <c r="H264" s="47" t="s">
         <v>137</v>
@@ -13135,7 +13135,7 @@
     </row>
     <row r="265" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A265" s="51" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
       <c r="H265" s="47" t="s">
         <v>137</v>
@@ -13525,7 +13525,7 @@
         <v>82</v>
       </c>
       <c r="V279" s="57" t="s">
-        <v>1325</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="280" spans="1:22" x14ac:dyDescent="0.25">
@@ -13634,7 +13634,7 @@
     </row>
     <row r="284" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A284" s="51" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
       <c r="H284" s="47" t="s">
         <v>138</v>
@@ -13669,7 +13669,7 @@
     </row>
     <row r="285" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A285" s="51" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
       <c r="H285" s="47" t="s">
         <v>138</v>
@@ -13924,7 +13924,7 @@
     </row>
     <row r="295" spans="4:22" x14ac:dyDescent="0.25">
       <c r="F295" s="54" t="s">
-        <v>1310</v>
+        <v>1309</v>
       </c>
       <c r="I295" s="8" t="s">
         <v>23</v>
@@ -13951,7 +13951,7 @@
     </row>
     <row r="296" spans="4:22" x14ac:dyDescent="0.25">
       <c r="F296" s="54" t="s">
-        <v>1310</v>
+        <v>1309</v>
       </c>
       <c r="I296" s="8" t="s">
         <v>23</v>
@@ -13982,7 +13982,7 @@
         <v>127</v>
       </c>
       <c r="F297" s="54" t="s">
-        <v>1310</v>
+        <v>1309</v>
       </c>
       <c r="I297" s="8" t="s">
         <v>23</v>
@@ -14012,7 +14012,7 @@
     </row>
     <row r="298" spans="4:22" x14ac:dyDescent="0.25">
       <c r="F298" s="54" t="s">
-        <v>1310</v>
+        <v>1309</v>
       </c>
       <c r="I298" s="8" t="s">
         <v>23</v>
@@ -15834,7 +15834,7 @@
     </row>
     <row r="368" spans="4:22" x14ac:dyDescent="0.25">
       <c r="D368" s="48" t="s">
-        <v>1304</v>
+        <v>1303</v>
       </c>
       <c r="H368" s="47" t="s">
         <v>140</v>
@@ -20368,7 +20368,7 @@
         <v>82</v>
       </c>
       <c r="V544" s="59" t="s">
-        <v>1322</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="545" spans="9:22" x14ac:dyDescent="0.25">
@@ -22422,7 +22422,7 @@
         <v>95</v>
       </c>
       <c r="V625" s="59" t="s">
-        <v>1323</v>
+        <v>1322</v>
       </c>
     </row>
     <row r="626" spans="1:22" x14ac:dyDescent="0.25">
@@ -22905,7 +22905,7 @@
         <v>82</v>
       </c>
       <c r="V643" s="57" t="s">
-        <v>1329</v>
+        <v>1328</v>
       </c>
     </row>
     <row r="644" spans="5:22" x14ac:dyDescent="0.25">
@@ -23114,10 +23114,10 @@
     </row>
     <row r="652" spans="5:22" x14ac:dyDescent="0.25">
       <c r="E652" s="54" t="s">
+        <v>1308</v>
+      </c>
+      <c r="F652" s="54" t="s">
         <v>1309</v>
-      </c>
-      <c r="F652" s="54" t="s">
-        <v>1310</v>
       </c>
       <c r="I652" s="8" t="s">
         <v>30</v>
@@ -23144,10 +23144,10 @@
     </row>
     <row r="653" spans="5:22" x14ac:dyDescent="0.25">
       <c r="E653" s="54" t="s">
+        <v>1308</v>
+      </c>
+      <c r="F653" s="54" t="s">
         <v>1309</v>
-      </c>
-      <c r="F653" s="54" t="s">
-        <v>1310</v>
       </c>
       <c r="I653" s="8" t="s">
         <v>30</v>
@@ -23385,7 +23385,7 @@
         <v>82</v>
       </c>
       <c r="V661" s="57" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="662" spans="8:22" x14ac:dyDescent="0.25">
@@ -24707,7 +24707,7 @@
     </row>
     <row r="713" spans="5:22" x14ac:dyDescent="0.25">
       <c r="E713" s="54" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="H713" s="47" t="s">
         <v>146</v>
@@ -24745,7 +24745,7 @@
     </row>
     <row r="714" spans="5:22" x14ac:dyDescent="0.25">
       <c r="E714" s="54" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="H714" s="47" t="s">
         <v>146</v>
@@ -24783,7 +24783,7 @@
     </row>
     <row r="715" spans="5:22" x14ac:dyDescent="0.25">
       <c r="E715" s="54" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="H715" s="47" t="s">
         <v>146</v>
@@ -24816,7 +24816,7 @@
     </row>
     <row r="716" spans="5:22" x14ac:dyDescent="0.25">
       <c r="E716" s="54" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="H716" s="47" t="s">
         <v>146</v>
@@ -29029,7 +29029,7 @@
         <v>11</v>
       </c>
       <c r="N880" s="5" t="s">
-        <v>1320</v>
+        <v>1319</v>
       </c>
       <c r="O880" s="2" t="s">
         <v>0</v>
@@ -32642,7 +32642,7 @@
         <v>82</v>
       </c>
       <c r="V1023" s="57" t="s">
-        <v>1326</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="1024" spans="4:22" x14ac:dyDescent="0.25">
@@ -32822,7 +32822,7 @@
         <v>123</v>
       </c>
       <c r="D1030" s="48" t="s">
-        <v>1305</v>
+        <v>1304</v>
       </c>
       <c r="H1030" s="47" t="s">
         <v>150</v>
@@ -32916,7 +32916,7 @@
     </row>
     <row r="1033" spans="1:22" x14ac:dyDescent="0.25">
       <c r="D1033" s="48" t="s">
-        <v>1305</v>
+        <v>1304</v>
       </c>
       <c r="H1033" s="47" t="s">
         <v>150</v>
@@ -33013,7 +33013,7 @@
         <v>82</v>
       </c>
       <c r="V1035" s="57" t="s">
-        <v>1327</v>
+        <v>1326</v>
       </c>
     </row>
     <row r="1036" spans="1:22" x14ac:dyDescent="0.25">
@@ -34805,7 +34805,7 @@
     </row>
     <row r="1106" spans="1:22" x14ac:dyDescent="0.25">
       <c r="F1106" s="54" t="s">
-        <v>1314</v>
+        <v>1313</v>
       </c>
       <c r="G1106" s="47" t="s">
         <v>133</v>
@@ -34835,10 +34835,10 @@
     </row>
     <row r="1107" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B1107" s="54" t="s">
-        <v>1308</v>
+        <v>1307</v>
       </c>
       <c r="F1107" s="54" t="s">
-        <v>1314</v>
+        <v>1313</v>
       </c>
       <c r="G1107" s="47" t="s">
         <v>133</v>
@@ -35213,7 +35213,7 @@
         <v>64</v>
       </c>
       <c r="N1121" s="5" t="s">
-        <v>1328</v>
+        <v>1327</v>
       </c>
       <c r="O1121" s="2" t="s">
         <v>0</v>
@@ -36071,7 +36071,7 @@
     </row>
     <row r="1155" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1155" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="E1155" s="47" t="s">
         <v>131</v>
@@ -36102,7 +36102,7 @@
     </row>
     <row r="1156" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1156" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="E1156" s="47" t="s">
         <v>131</v>
@@ -36139,7 +36139,7 @@
     </row>
     <row r="1157" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1157" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="H1157" s="47" t="s">
         <v>153</v>
@@ -36169,7 +36169,7 @@
     </row>
     <row r="1158" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1158" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="H1158" s="47" t="s">
         <v>153</v>
@@ -36202,7 +36202,7 @@
     </row>
     <row r="1159" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1159" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1159" s="8" t="s">
         <v>41</v>
@@ -36230,7 +36230,7 @@
     </row>
     <row r="1160" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1160" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1160" s="8" t="s">
         <v>41</v>
@@ -36257,7 +36257,7 @@
     </row>
     <row r="1161" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1161" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1161" s="8" t="s">
         <v>41</v>
@@ -36285,7 +36285,7 @@
     </row>
     <row r="1162" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1162" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1162" s="8" t="s">
         <v>41</v>
@@ -36312,7 +36312,7 @@
     </row>
     <row r="1163" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1163" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1163" s="8" t="s">
         <v>41</v>
@@ -36339,7 +36339,7 @@
     </row>
     <row r="1164" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1164" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1164" s="8" t="s">
         <v>41</v>
@@ -36366,7 +36366,7 @@
     </row>
     <row r="1165" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1165" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1165" s="8" t="s">
         <v>41</v>
@@ -36398,7 +36398,7 @@
     </row>
     <row r="1166" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1166" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1166" s="8" t="s">
         <v>41</v>
@@ -36425,7 +36425,7 @@
     </row>
     <row r="1167" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1167" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1167" s="8" t="s">
         <v>41</v>
@@ -36452,7 +36452,7 @@
     </row>
     <row r="1168" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1168" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1168" s="8" t="s">
         <v>41</v>
@@ -36480,7 +36480,7 @@
     </row>
     <row r="1169" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1169" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1169" s="8" t="s">
         <v>41</v>
@@ -36507,7 +36507,7 @@
     </row>
     <row r="1170" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1170" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1170" s="8" t="s">
         <v>41</v>
@@ -36539,7 +36539,7 @@
     </row>
     <row r="1171" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1171" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1171" s="8" t="s">
         <v>41</v>
@@ -36566,7 +36566,7 @@
     </row>
     <row r="1172" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1172" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1172" s="8" t="s">
         <v>41</v>
@@ -36593,7 +36593,7 @@
     </row>
     <row r="1173" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1173" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1173" s="8" t="s">
         <v>41</v>
@@ -36625,7 +36625,7 @@
     </row>
     <row r="1174" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1174" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1174" s="8" t="s">
         <v>41</v>
@@ -36652,7 +36652,7 @@
     </row>
     <row r="1175" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1175" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1175" s="8" t="s">
         <v>41</v>
@@ -36679,7 +36679,7 @@
     </row>
     <row r="1176" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1176" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1176" s="8" t="s">
         <v>41</v>
@@ -36711,7 +36711,7 @@
     </row>
     <row r="1177" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1177" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1177" s="8" t="s">
         <v>41</v>
@@ -36741,7 +36741,7 @@
     </row>
     <row r="1178" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1178" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1178" s="8" t="s">
         <v>41</v>
@@ -36768,7 +36768,7 @@
     </row>
     <row r="1179" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1179" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1179" s="8" t="s">
         <v>41</v>
@@ -36795,7 +36795,7 @@
     </row>
     <row r="1180" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1180" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1180" s="8" t="s">
         <v>41</v>
@@ -36822,7 +36822,7 @@
     </row>
     <row r="1181" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1181" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1181" s="8" t="s">
         <v>41</v>
@@ -36849,7 +36849,7 @@
     </row>
     <row r="1182" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1182" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1182" s="8" t="s">
         <v>41</v>
@@ -36876,7 +36876,7 @@
     </row>
     <row r="1183" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1183" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1183" s="8" t="s">
         <v>41</v>
@@ -36908,7 +36908,7 @@
     </row>
     <row r="1184" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1184" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1184" s="8" t="s">
         <v>41</v>
@@ -36940,7 +36940,7 @@
     </row>
     <row r="1185" spans="1:22" x14ac:dyDescent="0.25">
       <c r="C1185" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1185" s="8" t="s">
         <v>41</v>
@@ -36967,7 +36967,7 @@
     </row>
     <row r="1186" spans="1:22" x14ac:dyDescent="0.25">
       <c r="C1186" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1186" s="8" t="s">
         <v>41</v>
@@ -36994,7 +36994,7 @@
     </row>
     <row r="1187" spans="1:22" x14ac:dyDescent="0.25">
       <c r="C1187" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1187" s="8" t="s">
         <v>41</v>
@@ -37021,7 +37021,7 @@
     </row>
     <row r="1188" spans="1:22" x14ac:dyDescent="0.25">
       <c r="C1188" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1188" s="8" t="s">
         <v>41</v>
@@ -37048,7 +37048,7 @@
     </row>
     <row r="1189" spans="1:22" x14ac:dyDescent="0.25">
       <c r="C1189" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1189" s="8" t="s">
         <v>41</v>
@@ -37080,7 +37080,7 @@
     </row>
     <row r="1190" spans="1:22" x14ac:dyDescent="0.25">
       <c r="C1190" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1190" s="8" t="s">
         <v>41</v>
@@ -37107,7 +37107,7 @@
     </row>
     <row r="1191" spans="1:22" x14ac:dyDescent="0.25">
       <c r="C1191" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1191" s="8" t="s">
         <v>41</v>
@@ -37139,7 +37139,7 @@
     </row>
     <row r="1192" spans="1:22" x14ac:dyDescent="0.25">
       <c r="C1192" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1192" s="8" t="s">
         <v>41</v>
@@ -37166,7 +37166,7 @@
     </row>
     <row r="1193" spans="1:22" x14ac:dyDescent="0.25">
       <c r="C1193" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1193" s="8" t="s">
         <v>41</v>
@@ -37193,7 +37193,7 @@
     </row>
     <row r="1194" spans="1:22" x14ac:dyDescent="0.25">
       <c r="C1194" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1194" s="8" t="s">
         <v>41</v>
@@ -37223,10 +37223,10 @@
     </row>
     <row r="1195" spans="1:22" x14ac:dyDescent="0.25">
       <c r="C1195" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="F1195" s="54" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="I1195" s="8" t="s">
         <v>41</v>
@@ -37250,7 +37250,7 @@
         <v>829</v>
       </c>
       <c r="S1195" s="41" t="s">
-        <v>1321</v>
+        <v>1320</v>
       </c>
       <c r="T1195" s="2" t="s">
         <v>113</v>
@@ -37262,10 +37262,10 @@
         <v>123</v>
       </c>
       <c r="C1196" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="F1196" s="54" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="I1196" s="8" t="s">
         <v>41</v>
@@ -37292,7 +37292,7 @@
     </row>
     <row r="1197" spans="1:22" x14ac:dyDescent="0.25">
       <c r="C1197" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1197" s="8" t="s">
         <v>41</v>
@@ -37324,7 +37324,7 @@
     </row>
     <row r="1198" spans="1:22" x14ac:dyDescent="0.25">
       <c r="C1198" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1198" s="8" t="s">
         <v>41</v>
@@ -37351,7 +37351,7 @@
     </row>
     <row r="1199" spans="1:22" x14ac:dyDescent="0.25">
       <c r="C1199" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1199" s="8" t="s">
         <v>41</v>
@@ -37378,7 +37378,7 @@
     </row>
     <row r="1200" spans="1:22" x14ac:dyDescent="0.25">
       <c r="C1200" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1200" s="8" t="s">
         <v>41</v>
@@ -37405,7 +37405,7 @@
     </row>
     <row r="1201" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1201" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1201" s="8" t="s">
         <v>41</v>
@@ -37437,7 +37437,7 @@
     </row>
     <row r="1202" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1202" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1202" s="8" t="s">
         <v>41</v>
@@ -37465,7 +37465,7 @@
     </row>
     <row r="1203" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1203" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="I1203" s="8" t="s">
         <v>41</v>
@@ -37492,7 +37492,7 @@
     </row>
     <row r="1204" spans="3:22" x14ac:dyDescent="0.25">
       <c r="C1204" s="49" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="H1204" s="47" t="s">
         <v>154</v>
@@ -40288,8 +40288,8 @@
       <c r="P1307" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="V1307" s="35" t="s">
-        <v>1243</v>
+      <c r="V1307" s="57" t="s">
+        <v>1329</v>
       </c>
     </row>
     <row r="1308" spans="8:22" x14ac:dyDescent="0.25">
@@ -40390,7 +40390,7 @@
         <v>0</v>
       </c>
       <c r="V1311" s="14" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
     </row>
     <row r="1312" spans="8:22" x14ac:dyDescent="0.25">
@@ -40443,7 +40443,7 @@
         <v>0</v>
       </c>
       <c r="V1313" s="14" t="s">
-        <v>1245</v>
+        <v>1244</v>
       </c>
     </row>
     <row r="1314" spans="9:22" x14ac:dyDescent="0.25">
@@ -40549,7 +40549,7 @@
         <v>0</v>
       </c>
       <c r="V1317" s="14" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="1318" spans="9:22" x14ac:dyDescent="0.25">
@@ -40650,7 +40650,7 @@
         <v>0</v>
       </c>
       <c r="V1321" s="14" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="1322" spans="9:22" x14ac:dyDescent="0.25">
@@ -40679,7 +40679,7 @@
         <v>82</v>
       </c>
       <c r="V1322" s="31" t="s">
-        <v>1248</v>
+        <v>1247</v>
       </c>
     </row>
     <row r="1323" spans="9:22" x14ac:dyDescent="0.25">
@@ -40708,7 +40708,7 @@
         <v>89</v>
       </c>
       <c r="T1323" s="2" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
       <c r="V1323" s="14"/>
     </row>
@@ -40862,7 +40862,7 @@
         <v>82</v>
       </c>
       <c r="V1329" s="28" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
     </row>
     <row r="1330" spans="4:22" x14ac:dyDescent="0.25">
@@ -41017,7 +41017,7 @@
         <v>181</v>
       </c>
       <c r="N1335" s="55" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
       <c r="O1335" s="1" t="s">
         <v>102</v>
@@ -41138,7 +41138,7 @@
         <v>0</v>
       </c>
       <c r="V1339" s="14" t="s">
-        <v>1250</v>
+        <v>1249</v>
       </c>
     </row>
     <row r="1340" spans="4:22" x14ac:dyDescent="0.25">
@@ -41251,7 +41251,7 @@
         <v>0</v>
       </c>
       <c r="V1343" s="14" t="s">
-        <v>1251</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="1344" spans="4:22" x14ac:dyDescent="0.25">
@@ -41280,7 +41280,7 @@
         <v>0</v>
       </c>
       <c r="V1344" s="14" t="s">
-        <v>1252</v>
+        <v>1251</v>
       </c>
     </row>
     <row r="1345" spans="9:22" x14ac:dyDescent="0.25">
@@ -41309,7 +41309,7 @@
         <v>82</v>
       </c>
       <c r="V1345" s="28" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
     </row>
     <row r="1346" spans="9:22" x14ac:dyDescent="0.25">
@@ -41582,7 +41582,7 @@
         <v>82</v>
       </c>
       <c r="V1356" s="35" t="s">
-        <v>1254</v>
+        <v>1253</v>
       </c>
     </row>
     <row r="1357" spans="9:22" x14ac:dyDescent="0.25">
@@ -41660,7 +41660,7 @@
         <v>0</v>
       </c>
       <c r="V1359" s="14" t="s">
-        <v>1255</v>
+        <v>1254</v>
       </c>
     </row>
     <row r="1360" spans="9:22" x14ac:dyDescent="0.25">
@@ -41689,7 +41689,7 @@
         <v>0</v>
       </c>
       <c r="V1360" s="14" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="1361" spans="4:22" x14ac:dyDescent="0.25">
@@ -41721,7 +41721,7 @@
         <v>82</v>
       </c>
       <c r="V1361" s="14" t="s">
-        <v>1257</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="1362" spans="4:22" x14ac:dyDescent="0.25">
@@ -41802,7 +41802,7 @@
         <v>82</v>
       </c>
       <c r="V1364" s="14" t="s">
-        <v>1258</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="1365" spans="4:22" x14ac:dyDescent="0.25">
@@ -42047,7 +42047,7 @@
         <v>82</v>
       </c>
       <c r="V1373" s="14" t="s">
-        <v>1259</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="1374" spans="4:22" x14ac:dyDescent="0.25">
@@ -42100,7 +42100,7 @@
         <v>0</v>
       </c>
       <c r="V1375" s="14" t="s">
-        <v>1260</v>
+        <v>1259</v>
       </c>
     </row>
     <row r="1376" spans="4:22" x14ac:dyDescent="0.25">
@@ -42135,7 +42135,7 @@
       <c r="T1376" s="43"/>
       <c r="U1376" s="43"/>
       <c r="V1376" s="14" t="s">
-        <v>1261</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="1377" spans="8:22" x14ac:dyDescent="0.25">
@@ -42273,7 +42273,7 @@
         <v>82</v>
       </c>
       <c r="V1381" s="14" t="s">
-        <v>1262</v>
+        <v>1261</v>
       </c>
     </row>
     <row r="1382" spans="8:22" x14ac:dyDescent="0.25">
@@ -42449,7 +42449,7 @@
         <v>82</v>
       </c>
       <c r="V1388" s="28" t="s">
-        <v>1263</v>
+        <v>1262</v>
       </c>
     </row>
     <row r="1389" spans="8:22" x14ac:dyDescent="0.25">
@@ -42529,7 +42529,7 @@
         <v>82</v>
       </c>
       <c r="V1391" s="14" t="s">
-        <v>1264</v>
+        <v>1263</v>
       </c>
     </row>
     <row r="1392" spans="8:22" x14ac:dyDescent="0.25">
@@ -42683,7 +42683,7 @@
         <v>0</v>
       </c>
       <c r="V1397" s="14" t="s">
-        <v>1265</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="1398" spans="9:22" x14ac:dyDescent="0.25">
@@ -42760,7 +42760,7 @@
         <v>82</v>
       </c>
       <c r="V1400" s="28" t="s">
-        <v>1266</v>
+        <v>1265</v>
       </c>
     </row>
     <row r="1401" spans="9:22" x14ac:dyDescent="0.25">
@@ -42870,7 +42870,7 @@
         <v>0</v>
       </c>
       <c r="V1404" s="14" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
     </row>
     <row r="1405" spans="9:22" x14ac:dyDescent="0.25">
@@ -42997,7 +42997,7 @@
         <v>82</v>
       </c>
       <c r="V1409" s="14" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="1410" spans="9:22" x14ac:dyDescent="0.25">
@@ -43101,7 +43101,7 @@
         <v>0</v>
       </c>
       <c r="V1413" s="14" t="s">
-        <v>1269</v>
+        <v>1268</v>
       </c>
     </row>
     <row r="1414" spans="9:22" x14ac:dyDescent="0.25">
@@ -43225,7 +43225,7 @@
         <v>0</v>
       </c>
       <c r="V1418" s="8" t="s">
-        <v>1270</v>
+        <v>1269</v>
       </c>
     </row>
     <row r="1419" spans="9:22" x14ac:dyDescent="0.25">
@@ -43282,7 +43282,7 @@
         <v>95</v>
       </c>
       <c r="V1420" s="35" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
     </row>
     <row r="1421" spans="9:22" x14ac:dyDescent="0.25">
@@ -43408,7 +43408,7 @@
         <v>0</v>
       </c>
       <c r="V1425" s="14" t="s">
-        <v>1272</v>
+        <v>1271</v>
       </c>
     </row>
     <row r="1426" spans="8:22" x14ac:dyDescent="0.25">
@@ -43659,7 +43659,7 @@
         <v>0</v>
       </c>
       <c r="V1435" s="14" t="s">
-        <v>1273</v>
+        <v>1272</v>
       </c>
     </row>
     <row r="1436" spans="8:22" x14ac:dyDescent="0.25">
@@ -43691,7 +43691,7 @@
         <v>82</v>
       </c>
       <c r="V1436" s="28" t="s">
-        <v>1274</v>
+        <v>1273</v>
       </c>
     </row>
     <row r="1437" spans="8:22" x14ac:dyDescent="0.25">
@@ -43777,7 +43777,7 @@
         <v>0</v>
       </c>
       <c r="V1439" s="14" t="s">
-        <v>1275</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="1440" spans="8:22" x14ac:dyDescent="0.25">
@@ -43806,7 +43806,7 @@
         <v>0</v>
       </c>
       <c r="V1440" s="14" t="s">
-        <v>1276</v>
+        <v>1275</v>
       </c>
     </row>
     <row r="1441" spans="1:22" x14ac:dyDescent="0.25">
@@ -43883,7 +43883,7 @@
         <v>0</v>
       </c>
       <c r="V1443" s="14" t="s">
-        <v>1277</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="1444" spans="1:22" x14ac:dyDescent="0.25">
@@ -43936,7 +43936,7 @@
         <v>82</v>
       </c>
       <c r="V1445" s="32" t="s">
-        <v>1278</v>
+        <v>1277</v>
       </c>
     </row>
     <row r="1446" spans="1:22" x14ac:dyDescent="0.25">
@@ -44088,7 +44088,7 @@
         <v>0</v>
       </c>
       <c r="V1451" s="14" t="s">
-        <v>1279</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="1452" spans="1:22" x14ac:dyDescent="0.25">
@@ -44117,7 +44117,7 @@
         <v>82</v>
       </c>
       <c r="V1452" s="28" t="s">
-        <v>1280</v>
+        <v>1279</v>
       </c>
     </row>
     <row r="1453" spans="1:22" x14ac:dyDescent="0.25">
@@ -44197,7 +44197,7 @@
     </row>
     <row r="1456" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1456" s="51" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
       <c r="H1456" s="47" t="s">
         <v>160</v>
@@ -44230,7 +44230,7 @@
     </row>
     <row r="1457" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1457" s="51" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
       <c r="H1457" s="47" t="s">
         <v>160</v>
@@ -44314,7 +44314,7 @@
         <v>82</v>
       </c>
       <c r="V1459" s="28" t="s">
-        <v>1281</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="1460" spans="1:22" x14ac:dyDescent="0.25">
@@ -44394,7 +44394,7 @@
         <v>0</v>
       </c>
       <c r="V1462" s="14" t="s">
-        <v>1282</v>
+        <v>1281</v>
       </c>
     </row>
     <row r="1463" spans="1:22" x14ac:dyDescent="0.25">
@@ -44677,7 +44677,7 @@
         <v>82</v>
       </c>
       <c r="V1473" s="14" t="s">
-        <v>1283</v>
+        <v>1282</v>
       </c>
     </row>
     <row r="1474" spans="6:22" x14ac:dyDescent="0.25">
@@ -44706,7 +44706,7 @@
         <v>0</v>
       </c>
       <c r="V1474" s="14" t="s">
-        <v>1284</v>
+        <v>1283</v>
       </c>
     </row>
     <row r="1475" spans="6:22" x14ac:dyDescent="0.25">
@@ -44735,7 +44735,7 @@
         <v>0</v>
       </c>
       <c r="V1475" s="14" t="s">
-        <v>1285</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="1476" spans="6:22" x14ac:dyDescent="0.25">
@@ -44764,7 +44764,7 @@
         <v>0</v>
       </c>
       <c r="V1476" s="14" t="s">
-        <v>1286</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="1477" spans="6:22" x14ac:dyDescent="0.25">
@@ -44793,7 +44793,7 @@
         <v>82</v>
       </c>
       <c r="V1477" s="8" t="s">
-        <v>1287</v>
+        <v>1286</v>
       </c>
     </row>
     <row r="1478" spans="6:22" x14ac:dyDescent="0.25">
@@ -44873,12 +44873,12 @@
         <v>95</v>
       </c>
       <c r="V1480" s="28" t="s">
-        <v>1288</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="1481" spans="6:22" x14ac:dyDescent="0.25">
       <c r="F1481" s="54" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="H1481" s="47" t="s">
         <v>161</v>
@@ -44908,7 +44908,7 @@
     </row>
     <row r="1482" spans="6:22" x14ac:dyDescent="0.25">
       <c r="F1482" s="54" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="H1482" s="47" t="s">
         <v>161</v>
@@ -44965,7 +44965,7 @@
         <v>15</v>
       </c>
       <c r="V1483" s="26" t="s">
-        <v>1289</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="1484" spans="6:22" x14ac:dyDescent="0.25">
@@ -45027,7 +45027,7 @@
         <v>0</v>
       </c>
       <c r="V1485" s="14" t="s">
-        <v>1290</v>
+        <v>1289</v>
       </c>
     </row>
     <row r="1486" spans="6:22" x14ac:dyDescent="0.25">
@@ -45160,7 +45160,7 @@
         <v>82</v>
       </c>
       <c r="V1490" s="28" t="s">
-        <v>1291</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="1491" spans="8:22" x14ac:dyDescent="0.25">
@@ -45261,7 +45261,7 @@
         <v>0</v>
       </c>
       <c r="V1494" s="60" t="s">
-        <v>1324</v>
+        <v>1323</v>
       </c>
     </row>
     <row r="1495" spans="8:22" x14ac:dyDescent="0.25">
@@ -45482,7 +45482,7 @@
         <v>122</v>
       </c>
       <c r="V1502" s="28" t="s">
-        <v>1292</v>
+        <v>1291</v>
       </c>
     </row>
     <row r="1503" spans="8:22" x14ac:dyDescent="0.25">
@@ -45783,7 +45783,7 @@
         <v>82</v>
       </c>
       <c r="V1514" s="28" t="s">
-        <v>1293</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="1515" spans="5:22" x14ac:dyDescent="0.25">
@@ -45812,7 +45812,7 @@
     </row>
     <row r="1516" spans="5:22" x14ac:dyDescent="0.25">
       <c r="F1516" s="54" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
       <c r="I1516" s="8" t="s">
         <v>48</v>
@@ -45839,7 +45839,7 @@
     </row>
     <row r="1517" spans="5:22" x14ac:dyDescent="0.25">
       <c r="F1517" s="54" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
       <c r="I1517" s="8" t="s">
         <v>48</v>
@@ -45866,7 +45866,7 @@
         <v>0</v>
       </c>
       <c r="V1517" s="14" t="s">
-        <v>1294</v>
+        <v>1293</v>
       </c>
     </row>
     <row r="1518" spans="5:22" x14ac:dyDescent="0.25">
@@ -45874,7 +45874,7 @@
         <v>131</v>
       </c>
       <c r="F1518" s="54" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
       <c r="I1518" s="8" t="s">
         <v>48</v>
@@ -45904,7 +45904,7 @@
         <v>99</v>
       </c>
       <c r="V1518" s="26" t="s">
-        <v>1295</v>
+        <v>1294</v>
       </c>
     </row>
     <row r="1519" spans="5:22" x14ac:dyDescent="0.25">
@@ -45912,7 +45912,7 @@
         <v>131</v>
       </c>
       <c r="F1519" s="54" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
       <c r="I1519" s="8" t="s">
         <v>48</v>
@@ -45966,7 +45966,7 @@
         <v>82</v>
       </c>
       <c r="V1520" s="14" t="s">
-        <v>1296</v>
+        <v>1295</v>
       </c>
     </row>
     <row r="1521" spans="1:22" x14ac:dyDescent="0.25">
@@ -46349,7 +46349,7 @@
         <v>82</v>
       </c>
       <c r="V1535" s="36" t="s">
-        <v>1297</v>
+        <v>1296</v>
       </c>
     </row>
     <row r="1536" spans="1:22" x14ac:dyDescent="0.25">
@@ -46579,7 +46579,7 @@
         <v>82</v>
       </c>
       <c r="V1544" s="28" t="s">
-        <v>1298</v>
+        <v>1297</v>
       </c>
     </row>
     <row r="1545" spans="8:22" x14ac:dyDescent="0.25">
@@ -46766,7 +46766,7 @@
         <v>0</v>
       </c>
       <c r="V1551" s="14" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
     </row>
     <row r="1552" spans="8:22" x14ac:dyDescent="0.25">
@@ -46867,7 +46867,7 @@
         <v>82</v>
       </c>
       <c r="V1555" s="8" t="s">
-        <v>1300</v>
+        <v>1299</v>
       </c>
     </row>
     <row r="1556" spans="5:22" x14ac:dyDescent="0.25">
@@ -46947,7 +46947,7 @@
         <v>82</v>
       </c>
       <c r="V1558" s="14" t="s">
-        <v>1264</v>
+        <v>1263</v>
       </c>
     </row>
     <row r="1559" spans="5:22" x14ac:dyDescent="0.25">
@@ -47127,7 +47127,7 @@
         <v>82</v>
       </c>
       <c r="V1565" s="28" t="s">
-        <v>1301</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="1566" spans="5:22" x14ac:dyDescent="0.25">
@@ -47208,7 +47208,7 @@
         <v>95</v>
       </c>
       <c r="V1568" s="32" t="s">
-        <v>1302</v>
+        <v>1301</v>
       </c>
     </row>
   </sheetData>

</xml_diff>